<commit_message>
Added code for histogram reweighting and modified the EDM fit function
</commit_message>
<xml_diff>
--- a/Sheets/ThesisFitResults.xlsx
+++ b/Sheets/ThesisFitResults.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samuelgrant/Documents/gm2/EDM/Sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9185FD56-9C41-F448-B9B5-927BA9F55BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B09BBF-E082-5F46-BEB4-2C94D746A87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="860" yWindow="500" windowWidth="25780" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="860" yWindow="500" windowWidth="25780" windowHeight="17500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="UpdatedAcceptance2" sheetId="6" r:id="rId1"/>
-    <sheet name="UpdatedAcceptance1" sheetId="5" r:id="rId2"/>
-    <sheet name="ThesisFitResults" sheetId="1" r:id="rId3"/>
-    <sheet name="ChangingStats" sheetId="4" r:id="rId4"/>
-    <sheet name="UpdatedAcceptance" sheetId="2" r:id="rId5"/>
-    <sheet name="Testing" sheetId="3" r:id="rId6"/>
+    <sheet name="NoReweight" sheetId="7" r:id="rId1"/>
+    <sheet name="Run1Reweight" sheetId="8" r:id="rId2"/>
+    <sheet name="UpdatedAcceptance2" sheetId="6" r:id="rId3"/>
+    <sheet name="UpdatedAcceptance1" sheetId="5" r:id="rId4"/>
+    <sheet name="ThesisFitResults" sheetId="1" r:id="rId5"/>
+    <sheet name="ChangingStats" sheetId="4" r:id="rId6"/>
+    <sheet name="UpdatedAcceptance" sheetId="2" r:id="rId7"/>
+    <sheet name="Testing" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="34">
   <si>
     <t>Run-1a</t>
   </si>
@@ -133,6 +135,12 @@
   </si>
   <si>
     <t>Tilt [mrad]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> reweight_error</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> reweight_err</t>
   </si>
 </sst>
 </file>
@@ -637,13 +645,13 @@
     <xf numFmtId="11" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -998,6 +1006,1550 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1274229D-C95B-CA46-9CDE-E49016CF5741}">
+  <dimension ref="A1:M23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>0.40928199999999998</v>
+      </c>
+      <c r="C3">
+        <v>9.5316999999999999E-2</v>
+      </c>
+      <c r="D3">
+        <v>6.7000000000000002E-4</v>
+      </c>
+      <c r="E3">
+        <v>2.5600999999999999E-2</v>
+      </c>
+      <c r="F3">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G3">
+        <v>9.8966999999999999E-2</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1.3773700000000001E-18</v>
+      </c>
+      <c r="I3" s="1">
+        <v>3.0427299999999998E-19</v>
+      </c>
+      <c r="J3" s="1">
+        <v>2.1391E-21</v>
+      </c>
+      <c r="K3" s="1">
+        <v>8.1723200000000002E-20</v>
+      </c>
+      <c r="L3" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="M3" s="1">
+        <v>3.1592400000000002E-19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>7.7824000000000004E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.101839</v>
+      </c>
+      <c r="D4">
+        <v>4.2099999999999999E-4</v>
+      </c>
+      <c r="E4">
+        <v>-2.366E-3</v>
+      </c>
+      <c r="F4">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G4">
+        <v>0.102128</v>
+      </c>
+      <c r="H4" s="1">
+        <v>3.19286E-19</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3.2509100000000002E-19</v>
+      </c>
+      <c r="J4" s="1">
+        <v>1.34509E-21</v>
+      </c>
+      <c r="K4" s="1">
+        <v>-7.5528600000000002E-21</v>
+      </c>
+      <c r="L4" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="M4" s="1">
+        <v>3.2601499999999998E-19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0.25788499999999998</v>
+      </c>
+      <c r="C5">
+        <v>6.9957000000000005E-2</v>
+      </c>
+      <c r="D5">
+        <v>4.3600000000000003E-4</v>
+      </c>
+      <c r="E5">
+        <v>2.0939999999999999E-3</v>
+      </c>
+      <c r="F5">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G5">
+        <v>7.0369000000000001E-2</v>
+      </c>
+      <c r="H5" s="1">
+        <v>8.9407899999999997E-19</v>
+      </c>
+      <c r="I5" s="1">
+        <v>2.2331699999999998E-19</v>
+      </c>
+      <c r="J5" s="1">
+        <v>1.39073E-21</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6.6849300000000003E-21</v>
+      </c>
+      <c r="L5" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="M5" s="1">
+        <v>2.2463300000000001E-19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J8" t="s">
+        <v>7</v>
+      </c>
+      <c r="K8" t="s">
+        <v>8</v>
+      </c>
+      <c r="L8" t="s">
+        <v>9</v>
+      </c>
+      <c r="M8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>0.24920999999999999</v>
+      </c>
+      <c r="C9">
+        <v>8.1412999999999999E-2</v>
+      </c>
+      <c r="D9">
+        <v>4.08E-4</v>
+      </c>
+      <c r="E9">
+        <v>8.6560000000000005E-3</v>
+      </c>
+      <c r="F9">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G9">
+        <v>8.2280000000000006E-2</v>
+      </c>
+      <c r="H9" s="1">
+        <v>8.6806499999999997E-19</v>
+      </c>
+      <c r="I9" s="1">
+        <v>2.5988899999999999E-19</v>
+      </c>
+      <c r="J9" s="1">
+        <v>1.30158E-21</v>
+      </c>
+      <c r="K9" s="1">
+        <v>2.7631599999999999E-20</v>
+      </c>
+      <c r="L9" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="M9" s="1">
+        <v>2.6265500000000002E-19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>0.230905</v>
+      </c>
+      <c r="C10">
+        <v>8.7075E-2</v>
+      </c>
+      <c r="D10">
+        <v>4.8200000000000001E-4</v>
+      </c>
+      <c r="E10">
+        <v>1.6479999999999999E-3</v>
+      </c>
+      <c r="F10">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G10">
+        <v>8.7474999999999997E-2</v>
+      </c>
+      <c r="H10" s="1">
+        <v>8.0963099999999999E-19</v>
+      </c>
+      <c r="I10" s="1">
+        <v>2.7796399999999999E-19</v>
+      </c>
+      <c r="J10" s="1">
+        <v>1.53952E-21</v>
+      </c>
+      <c r="K10" s="1">
+        <v>5.2596299999999999E-21</v>
+      </c>
+      <c r="L10" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2.79239E-19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>0.24099100000000001</v>
+      </c>
+      <c r="C11">
+        <v>5.9782000000000002E-2</v>
+      </c>
+      <c r="D11">
+        <v>4.1599999999999997E-4</v>
+      </c>
+      <c r="E11">
+        <v>1.4339999999999999E-3</v>
+      </c>
+      <c r="F11">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G11">
+        <v>6.0356E-2</v>
+      </c>
+      <c r="H11" s="1">
+        <v>8.4182800000000002E-19</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1.90836E-19</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1.3267199999999999E-21</v>
+      </c>
+      <c r="K11" s="1">
+        <v>4.57806E-21</v>
+      </c>
+      <c r="L11" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1.9267E-19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>5</v>
+      </c>
+      <c r="I14" t="s">
+        <v>6</v>
+      </c>
+      <c r="J14" t="s">
+        <v>7</v>
+      </c>
+      <c r="K14" t="s">
+        <v>8</v>
+      </c>
+      <c r="L14" t="s">
+        <v>9</v>
+      </c>
+      <c r="M14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <v>0.49626300000000001</v>
+      </c>
+      <c r="C15">
+        <v>6.6790000000000002E-2</v>
+      </c>
+      <c r="D15">
+        <v>7.5699999999999997E-4</v>
+      </c>
+      <c r="E15">
+        <v>2.0955000000000001E-2</v>
+      </c>
+      <c r="F15">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G15">
+        <v>7.0487999999999995E-2</v>
+      </c>
+      <c r="H15" s="1">
+        <v>1.6786799999999999E-18</v>
+      </c>
+      <c r="I15" s="1">
+        <v>2.1320799999999999E-19</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2.4176200000000001E-21</v>
+      </c>
+      <c r="K15" s="1">
+        <v>6.68926E-20</v>
+      </c>
+      <c r="L15" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="M15" s="1">
+        <v>2.2501200000000002E-19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>0.40148699999999998</v>
+      </c>
+      <c r="C16">
+        <v>7.2070999999999996E-2</v>
+      </c>
+      <c r="D16">
+        <v>7.4700000000000005E-4</v>
+      </c>
+      <c r="E16">
+        <v>-9.0100000000000006E-3</v>
+      </c>
+      <c r="F16">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G16">
+        <v>7.3102E-2</v>
+      </c>
+      <c r="H16" s="1">
+        <v>1.3761400000000001E-18</v>
+      </c>
+      <c r="I16" s="1">
+        <v>2.3006700000000001E-19</v>
+      </c>
+      <c r="J16" s="1">
+        <v>2.3861600000000001E-21</v>
+      </c>
+      <c r="K16" s="1">
+        <v>-2.87614E-20</v>
+      </c>
+      <c r="L16" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2.3335799999999999E-19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>0.45368199999999997</v>
+      </c>
+      <c r="C17">
+        <v>4.9249000000000001E-2</v>
+      </c>
+      <c r="D17">
+        <v>7.2199999999999999E-4</v>
+      </c>
+      <c r="E17">
+        <v>1.7290000000000001E-3</v>
+      </c>
+      <c r="F17">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G17">
+        <v>4.9969E-2</v>
+      </c>
+      <c r="H17" s="1">
+        <v>1.5427499999999999E-18</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1.57213E-19</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2.3062199999999999E-21</v>
+      </c>
+      <c r="K17" s="1">
+        <v>5.5203200000000002E-21</v>
+      </c>
+      <c r="L17" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="M17" s="1">
+        <v>1.5951199999999999E-19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I20" t="s">
+        <v>6</v>
+      </c>
+      <c r="J20" t="s">
+        <v>7</v>
+      </c>
+      <c r="K20" t="s">
+        <v>8</v>
+      </c>
+      <c r="L20" t="s">
+        <v>9</v>
+      </c>
+      <c r="M20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21">
+        <v>0.34194400000000003</v>
+      </c>
+      <c r="C21">
+        <v>5.8612999999999998E-2</v>
+      </c>
+      <c r="D21">
+        <v>5.53E-4</v>
+      </c>
+      <c r="E21">
+        <v>1.3056999999999999E-2</v>
+      </c>
+      <c r="F21">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G21">
+        <v>6.0743999999999999E-2</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1.2009900000000001E-18</v>
+      </c>
+      <c r="I21" s="1">
+        <v>1.8710499999999999E-19</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1.7666099999999998E-21</v>
+      </c>
+      <c r="K21" s="1">
+        <v>4.1679700000000001E-20</v>
+      </c>
+      <c r="L21" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="M21" s="1">
+        <v>1.9390999999999999E-19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22">
+        <v>0.287055</v>
+      </c>
+      <c r="C22">
+        <v>6.3268000000000005E-2</v>
+      </c>
+      <c r="D22">
+        <v>5.9500000000000004E-4</v>
+      </c>
+      <c r="E22">
+        <v>5.7359999999999998E-3</v>
+      </c>
+      <c r="F22">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G22">
+        <v>6.4185000000000006E-2</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1.02577E-18</v>
+      </c>
+      <c r="I22" s="1">
+        <v>2.0196399999999999E-19</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1.8989099999999999E-21</v>
+      </c>
+      <c r="K22" s="1">
+        <v>1.8311300000000001E-20</v>
+      </c>
+      <c r="L22" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="M22" s="1">
+        <v>2.0489199999999999E-19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>0.31791000000000003</v>
+      </c>
+      <c r="C23">
+        <v>4.3221999999999997E-2</v>
+      </c>
+      <c r="D23">
+        <v>5.2300000000000003E-4</v>
+      </c>
+      <c r="E23">
+        <v>3.2100000000000002E-3</v>
+      </c>
+      <c r="F23">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G23">
+        <v>4.4298999999999998E-2</v>
+      </c>
+      <c r="H23" s="1">
+        <v>1.1242700000000001E-18</v>
+      </c>
+      <c r="I23" s="1">
+        <v>1.3797500000000001E-19</v>
+      </c>
+      <c r="J23" s="1">
+        <v>1.66972E-21</v>
+      </c>
+      <c r="K23" s="1">
+        <v>1.0248599999999999E-20</v>
+      </c>
+      <c r="L23" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="M23" s="1">
+        <v>1.4141199999999999E-19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C7B764-2406-AF47-AAA8-6C22321D8403}">
+  <dimension ref="A1:O23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>0.40928199999999998</v>
+      </c>
+      <c r="C3">
+        <v>9.5316999999999999E-2</v>
+      </c>
+      <c r="D3">
+        <v>6.7000000000000002E-4</v>
+      </c>
+      <c r="E3">
+        <v>2.5600999999999999E-2</v>
+      </c>
+      <c r="F3">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G3">
+        <v>9.8966999999999999E-2</v>
+      </c>
+      <c r="H3">
+        <v>6.8019999999999999E-3</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.3773700000000001E-18</v>
+      </c>
+      <c r="J3" s="1">
+        <v>3.0427299999999998E-19</v>
+      </c>
+      <c r="K3" s="1">
+        <v>2.1391E-21</v>
+      </c>
+      <c r="L3" s="1">
+        <v>8.1723200000000002E-20</v>
+      </c>
+      <c r="M3" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="N3" s="1">
+        <v>3.1592400000000002E-19</v>
+      </c>
+      <c r="O3" s="1">
+        <v>2.1713800000000001E-20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>7.7824000000000004E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.101839</v>
+      </c>
+      <c r="D4">
+        <v>4.2099999999999999E-4</v>
+      </c>
+      <c r="E4">
+        <v>-2.366E-3</v>
+      </c>
+      <c r="F4">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G4">
+        <v>0.102128</v>
+      </c>
+      <c r="H4">
+        <v>2.2369999999999998E-3</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3.19286E-19</v>
+      </c>
+      <c r="J4" s="1">
+        <v>3.2509100000000002E-19</v>
+      </c>
+      <c r="K4" s="1">
+        <v>1.34509E-21</v>
+      </c>
+      <c r="L4" s="1">
+        <v>-7.5528600000000002E-21</v>
+      </c>
+      <c r="M4" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="N4" s="1">
+        <v>3.2601499999999998E-19</v>
+      </c>
+      <c r="O4" s="1">
+        <v>7.1425000000000003E-21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>0.25788499999999998</v>
+      </c>
+      <c r="C5">
+        <v>6.9957000000000005E-2</v>
+      </c>
+      <c r="D5">
+        <v>4.3600000000000003E-4</v>
+      </c>
+      <c r="E5">
+        <v>2.0939999999999999E-3</v>
+      </c>
+      <c r="F5">
+        <v>7.2979999999999998E-3</v>
+      </c>
+      <c r="G5">
+        <v>7.0369000000000001E-2</v>
+      </c>
+      <c r="H5">
+        <v>4.9410000000000001E-3</v>
+      </c>
+      <c r="I5" s="1">
+        <v>8.9407899999999997E-19</v>
+      </c>
+      <c r="J5" s="1">
+        <v>2.2331699999999998E-19</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1.39073E-21</v>
+      </c>
+      <c r="L5" s="1">
+        <v>6.6849300000000003E-21</v>
+      </c>
+      <c r="M5" s="1">
+        <v>2.32968E-20</v>
+      </c>
+      <c r="N5" s="1">
+        <v>2.2463300000000001E-19</v>
+      </c>
+      <c r="O5" s="1">
+        <v>1.5774000000000001E-20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N8" t="s">
+        <v>10</v>
+      </c>
+      <c r="O8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>0.24920999999999999</v>
+      </c>
+      <c r="C9">
+        <v>8.1412999999999999E-2</v>
+      </c>
+      <c r="D9">
+        <v>4.08E-4</v>
+      </c>
+      <c r="E9">
+        <v>8.6560000000000005E-3</v>
+      </c>
+      <c r="F9">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G9">
+        <v>8.2280000000000006E-2</v>
+      </c>
+      <c r="H9">
+        <v>5.2030000000000002E-3</v>
+      </c>
+      <c r="I9" s="1">
+        <v>8.6806499999999997E-19</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2.5988899999999999E-19</v>
+      </c>
+      <c r="K9" s="1">
+        <v>1.30158E-21</v>
+      </c>
+      <c r="L9" s="1">
+        <v>2.7631599999999999E-20</v>
+      </c>
+      <c r="M9" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="N9" s="1">
+        <v>2.6265500000000002E-19</v>
+      </c>
+      <c r="O9" s="1">
+        <v>1.6608300000000001E-20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>0.230905</v>
+      </c>
+      <c r="C10">
+        <v>8.7075E-2</v>
+      </c>
+      <c r="D10">
+        <v>4.8200000000000001E-4</v>
+      </c>
+      <c r="E10">
+        <v>1.6479999999999999E-3</v>
+      </c>
+      <c r="F10">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G10">
+        <v>8.7474999999999997E-2</v>
+      </c>
+      <c r="H10">
+        <v>5.274E-3</v>
+      </c>
+      <c r="I10" s="1">
+        <v>8.0963099999999999E-19</v>
+      </c>
+      <c r="J10" s="1">
+        <v>2.7796399999999999E-19</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1.53952E-21</v>
+      </c>
+      <c r="L10" s="1">
+        <v>5.2596299999999999E-21</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="N10" s="1">
+        <v>2.79239E-19</v>
+      </c>
+      <c r="O10" s="1">
+        <v>1.6836699999999999E-20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>0.24099100000000001</v>
+      </c>
+      <c r="C11">
+        <v>5.9782000000000002E-2</v>
+      </c>
+      <c r="D11">
+        <v>4.1599999999999997E-4</v>
+      </c>
+      <c r="E11">
+        <v>1.4339999999999999E-3</v>
+      </c>
+      <c r="F11">
+        <v>8.1720000000000004E-3</v>
+      </c>
+      <c r="G11">
+        <v>6.0356E-2</v>
+      </c>
+      <c r="H11">
+        <v>5.2859999999999999E-3</v>
+      </c>
+      <c r="I11" s="1">
+        <v>8.4182800000000002E-19</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1.90836E-19</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1.3267199999999999E-21</v>
+      </c>
+      <c r="L11" s="1">
+        <v>4.57806E-21</v>
+      </c>
+      <c r="M11" s="1">
+        <v>2.6087E-20</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.9267E-19</v>
+      </c>
+      <c r="O11" s="1">
+        <v>1.6873700000000001E-20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I14" t="s">
+        <v>5</v>
+      </c>
+      <c r="J14" t="s">
+        <v>6</v>
+      </c>
+      <c r="K14" t="s">
+        <v>7</v>
+      </c>
+      <c r="L14" t="s">
+        <v>8</v>
+      </c>
+      <c r="M14" t="s">
+        <v>9</v>
+      </c>
+      <c r="N14" t="s">
+        <v>10</v>
+      </c>
+      <c r="O14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <v>0.49626300000000001</v>
+      </c>
+      <c r="C15">
+        <v>6.6790000000000002E-2</v>
+      </c>
+      <c r="D15">
+        <v>7.5699999999999997E-4</v>
+      </c>
+      <c r="E15">
+        <v>2.0955000000000001E-2</v>
+      </c>
+      <c r="F15">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G15">
+        <v>7.0487999999999995E-2</v>
+      </c>
+      <c r="H15">
+        <v>1.0907E-2</v>
+      </c>
+      <c r="I15" s="1">
+        <v>1.6786799999999999E-18</v>
+      </c>
+      <c r="J15" s="1">
+        <v>2.1320799999999999E-19</v>
+      </c>
+      <c r="K15" s="1">
+        <v>2.4176200000000001E-21</v>
+      </c>
+      <c r="L15" s="1">
+        <v>6.68926E-20</v>
+      </c>
+      <c r="M15" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="N15" s="1">
+        <v>2.2501200000000002E-19</v>
+      </c>
+      <c r="O15" s="1">
+        <v>3.4818900000000001E-20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>0.40148699999999998</v>
+      </c>
+      <c r="C16">
+        <v>7.2070999999999996E-2</v>
+      </c>
+      <c r="D16">
+        <v>7.4700000000000005E-4</v>
+      </c>
+      <c r="E16">
+        <v>-9.0100000000000006E-3</v>
+      </c>
+      <c r="F16">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G16">
+        <v>7.3102E-2</v>
+      </c>
+      <c r="H16">
+        <v>1.0588999999999999E-2</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1.3761400000000001E-18</v>
+      </c>
+      <c r="J16" s="1">
+        <v>2.3006700000000001E-19</v>
+      </c>
+      <c r="K16" s="1">
+        <v>2.3861600000000001E-21</v>
+      </c>
+      <c r="L16" s="1">
+        <v>-2.87614E-20</v>
+      </c>
+      <c r="M16" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="N16" s="1">
+        <v>2.3335799999999999E-19</v>
+      </c>
+      <c r="O16" s="1">
+        <v>3.3804E-20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>0.45368199999999997</v>
+      </c>
+      <c r="C17">
+        <v>4.9249000000000001E-2</v>
+      </c>
+      <c r="D17">
+        <v>7.2199999999999999E-4</v>
+      </c>
+      <c r="E17">
+        <v>1.7290000000000001E-3</v>
+      </c>
+      <c r="F17">
+        <v>8.2430000000000003E-3</v>
+      </c>
+      <c r="G17">
+        <v>4.9969E-2</v>
+      </c>
+      <c r="H17">
+        <v>1.093E-2</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1.5427499999999999E-18</v>
+      </c>
+      <c r="J17" s="1">
+        <v>1.57213E-19</v>
+      </c>
+      <c r="K17" s="1">
+        <v>2.3062199999999999E-21</v>
+      </c>
+      <c r="L17" s="1">
+        <v>5.5203200000000002E-21</v>
+      </c>
+      <c r="M17" s="1">
+        <v>2.6313399999999999E-20</v>
+      </c>
+      <c r="N17" s="1">
+        <v>1.5951199999999999E-19</v>
+      </c>
+      <c r="O17" s="1">
+        <v>3.4892400000000001E-20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>32</v>
+      </c>
+      <c r="I20" t="s">
+        <v>5</v>
+      </c>
+      <c r="J20" t="s">
+        <v>6</v>
+      </c>
+      <c r="K20" t="s">
+        <v>7</v>
+      </c>
+      <c r="L20" t="s">
+        <v>8</v>
+      </c>
+      <c r="M20" t="s">
+        <v>9</v>
+      </c>
+      <c r="N20" t="s">
+        <v>10</v>
+      </c>
+      <c r="O20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21">
+        <v>0.34194400000000003</v>
+      </c>
+      <c r="C21">
+        <v>5.8612999999999998E-2</v>
+      </c>
+      <c r="D21">
+        <v>5.53E-4</v>
+      </c>
+      <c r="E21">
+        <v>1.3056999999999999E-2</v>
+      </c>
+      <c r="F21">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G21">
+        <v>6.0743999999999999E-2</v>
+      </c>
+      <c r="H21">
+        <v>7.9740000000000002E-3</v>
+      </c>
+      <c r="I21" s="1">
+        <v>1.2009900000000001E-18</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1.8710499999999999E-19</v>
+      </c>
+      <c r="K21" s="1">
+        <v>1.7666099999999998E-21</v>
+      </c>
+      <c r="L21" s="1">
+        <v>4.1679700000000001E-20</v>
+      </c>
+      <c r="M21" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="N21" s="1">
+        <v>1.9390999999999999E-19</v>
+      </c>
+      <c r="O21" s="1">
+        <v>2.5456000000000001E-20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22">
+        <v>0.287055</v>
+      </c>
+      <c r="C22">
+        <v>6.3268000000000005E-2</v>
+      </c>
+      <c r="D22">
+        <v>5.9500000000000004E-4</v>
+      </c>
+      <c r="E22">
+        <v>5.7359999999999998E-3</v>
+      </c>
+      <c r="F22">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G22">
+        <v>6.4185000000000006E-2</v>
+      </c>
+      <c r="H22">
+        <v>7.5490000000000002E-3</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1.02577E-18</v>
+      </c>
+      <c r="J22" s="1">
+        <v>2.0196399999999999E-19</v>
+      </c>
+      <c r="K22" s="1">
+        <v>1.8989099999999999E-21</v>
+      </c>
+      <c r="L22" s="1">
+        <v>1.8311300000000001E-20</v>
+      </c>
+      <c r="M22" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="N22" s="1">
+        <v>2.0489199999999999E-19</v>
+      </c>
+      <c r="O22" s="1">
+        <v>2.4096999999999999E-20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23">
+        <v>0.31791000000000003</v>
+      </c>
+      <c r="C23">
+        <v>4.3221999999999997E-2</v>
+      </c>
+      <c r="D23">
+        <v>5.2300000000000003E-4</v>
+      </c>
+      <c r="E23">
+        <v>3.2100000000000002E-3</v>
+      </c>
+      <c r="F23">
+        <v>9.1450000000000004E-3</v>
+      </c>
+      <c r="G23">
+        <v>4.4298999999999998E-2</v>
+      </c>
+      <c r="H23">
+        <v>7.9170000000000004E-3</v>
+      </c>
+      <c r="I23" s="1">
+        <v>1.1242700000000001E-18</v>
+      </c>
+      <c r="J23" s="1">
+        <v>1.3797500000000001E-19</v>
+      </c>
+      <c r="K23" s="1">
+        <v>1.66972E-21</v>
+      </c>
+      <c r="L23" s="1">
+        <v>1.0248599999999999E-20</v>
+      </c>
+      <c r="M23" s="1">
+        <v>2.91939E-20</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.4141199999999999E-19</v>
+      </c>
+      <c r="O23" s="1">
+        <v>2.5273399999999999E-20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{120B75E2-717F-A144-8F2D-53B72C32C006}">
   <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1582,10 +3134,10 @@
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C20" t="s">
@@ -1605,25 +3157,25 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="8" t="s">
         <v>10</v>
       </c>
       <c r="H21" t="s">
@@ -1646,7 +3198,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B22">
@@ -1687,7 +3239,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B23">
@@ -1728,7 +3280,7 @@
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B24">
@@ -1774,7 +3326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DDEFA7-60CA-0F48-9B06-175DAFEF0B41}">
   <dimension ref="A1:W33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1801,14 +3353,14 @@
       <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
-      <c r="S2" s="7"/>
-      <c r="T2" s="7"/>
-      <c r="U2" s="7"/>
-      <c r="V2" s="7"/>
-      <c r="W2" s="7"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1975,13 +3527,13 @@
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="D7" s="8"/>
+      <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
@@ -1993,7 +3545,7 @@
       <c r="E9" t="s">
         <v>2</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2162,13 +3714,13 @@
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="D14" s="8"/>
+      <c r="D14" s="7"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="8"/>
+      <c r="D15" s="7"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
@@ -2180,7 +3732,7 @@
       <c r="E16" t="s">
         <v>2</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2349,80 +3901,80 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D21" s="8"/>
+      <c r="D21" s="7"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D22" s="8"/>
+      <c r="D22" s="7"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9" t="s">
+      <c r="D23" s="8"/>
+      <c r="E23" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="11" t="s">
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I24" s="9" t="s">
+      <c r="I24" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J24" s="9" t="s">
+      <c r="J24" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="K24" s="9" t="s">
+      <c r="K24" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L24" s="9" t="s">
+      <c r="L24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="M24" s="9" t="s">
+      <c r="M24" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B25">
@@ -2463,7 +4015,7 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B26">
@@ -2504,7 +4056,7 @@
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B27">
@@ -2579,7 +4131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2605,22 +4157,22 @@
       <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7" t="s">
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="S2" s="7"/>
-      <c r="T2" s="7" t="s">
+      <c r="S2" s="11"/>
+      <c r="T2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="7"/>
-      <c r="V2" s="7" t="s">
+      <c r="U2" s="11"/>
+      <c r="V2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="W2" s="7"/>
+      <c r="W2" s="11"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -3486,7 +5038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21F37B0D-BB5E-F048-85FC-E6B6B5CA9825}">
   <dimension ref="A1:Q238"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -10494,7 +12046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809AB9B3-8782-1C47-A228-527379A36270}">
   <dimension ref="A1:AA32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11966,7 +13518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E1199F9-9CC5-574F-8FC3-3745086188F3}">
   <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>